<commit_message>
Update agent metadata and completion report
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/reports/P033r3_completion_report.xlsx
+++ b/reports/P033r3_completion_report.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Other pipe basis audit" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Downstream records" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Isolation checks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Production audit" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$30</definedName>
@@ -23,6 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Other pipe basis audit'!$A$1:$H$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Downstream records'!$A$1:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Isolation checks'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Production audit'!$A$1:$D$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -764,7 +766,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>NOT APPLIED — publish/schema migration and production flow remain separate</t>
+          <t>APPLIED AND VERIFIED — production revision batch 5</t>
         </is>
       </c>
     </row>
@@ -13128,7 +13130,6 @@
           <t>None explicitly referencing PPR</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
@@ -13174,7 +13175,6 @@
           <t>prayag-sales.com</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>90</v>
       </c>
@@ -13195,7 +13195,6 @@
           <t>No recorded activity event</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
@@ -13422,4 +13421,531 @@
   <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="53" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Before</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>After</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Successful published build</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Successful published build</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Revision batch</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Preview batch 5</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Applied batch 5</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>History rows</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>14342</v>
+      </c>
+      <c r="C4" t="n">
+        <v>14252</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PASS — exactly 90 deleted</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>History checksum</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4139138d8495b19c30b67677dcf08742</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>d4ba8d1ee1d5d73f02153f95f21abf7b</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Expected change</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Affected rows</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>270</v>
+      </c>
+      <c r="C6" t="n">
+        <v>180</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>May PPR rows</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>90</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>September PPR rows</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Codes with exactly two periods</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>90</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Workbook value mismatches</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Audit-note mismatches</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Unpriced PPR products</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>August current flags</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>90</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>February historical flags</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>90</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Staged updates / deletes</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>180 / 90</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Applied / deleted provenance events</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>180 / 90</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Competitor rows</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1915</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1915</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Competitor checksum</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>8acb3e044c47fc1421a71150186b4e4c</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>8acb3e044c47fc1421a71150186b4e4c</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>7141</v>
+      </c>
+      <c r="C20" t="n">
+        <v>7141</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Product checksum</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>a1be423219aacfdc19ec298e5c0a3c39</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>a1be423219aacfdc19ec298e5c0a3c39</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Prince median gap</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>+208.8074%</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>+2.9358%</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Prince range</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>+0.0393% to +3.9683%</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sample August values</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>P10A02=235; P10A03=324; P10G02=204</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Undo</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>One-action rollback available on production batch 5</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D25"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>